<commit_message>
fix(ui): degrade gracefully when live firewall function key is unavailable
- function_client returns local sample assessment when the function key is a placeholder or the function returns 401/403
- apply same guard to executive summary and excel report tools
- skip live assessment call in assessment_service when key is a placeholder
</commit_message>
<xml_diff>
--- a/ui/static/reports/PaloAlto_Assessment.xlsx
+++ b/ui/static/reports/PaloAlto_Assessment.xlsx
@@ -17,11 +17,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VPN" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Logging" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Administration" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backup" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zone Protection" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backup" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Compliance Results'!$A$1:$G$45</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Findings'!$A$1:$H$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Findings'!$A$1:$H$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -97,18 +98,18 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00D97706"/>
-    </font>
-    <font>
-      <b val="1"/>
       <color rgb="00B91C1C"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="0016A34A"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00D97706"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -143,12 +144,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FEE2E2"/>
         <bgColor rgb="00FEE2E2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-        <bgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -228,7 +223,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -268,16 +263,13 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -286,10 +278,10 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -688,7 +680,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>vmpafw01</t>
+          <t>edge-fw-01</t>
         </is>
       </c>
       <c r="C4" s="5" t="n"/>
@@ -702,7 +694,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>PA-VM</t>
+          <t>PA-3220</t>
         </is>
       </c>
       <c r="C5" s="5" t="n"/>
@@ -716,7 +708,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>10.2.10-h9</t>
+          <t>10.2.3</t>
         </is>
       </c>
       <c r="C6" s="5" t="n"/>
@@ -730,7 +722,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>007201234567</t>
         </is>
       </c>
       <c r="C7" s="5" t="n"/>
@@ -744,7 +736,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-14 03:17 IST</t>
+          <t>2026-08-14 04:39 IST</t>
         </is>
       </c>
       <c r="C8" s="5" t="n"/>
@@ -758,7 +750,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="C9" s="5" t="n"/>
@@ -788,7 +780,7 @@
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14">
@@ -798,7 +790,7 @@
         </is>
       </c>
       <c r="B14" s="11" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15">
@@ -808,7 +800,7 @@
         </is>
       </c>
       <c r="B15" s="12" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -848,7 +840,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -870,54 +862,72 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>administrators</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr"/>
+          <t>default_admin_disabled</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>management_allowed_ips</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr"/>
+          <t>https_enabled</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>https_enabled</t>
+          <t>management_acl_enabled</t>
         </is>
       </c>
       <c r="B4" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>ssh_enabled</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="b">
-        <v>1</v>
+          <t>admin_timeout_minutes</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>ntp_servers</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr"/>
+          <t>ntp_server_count</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
+          <t>snmp_version</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>v2c</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
           <t>panorama_managed</t>
         </is>
       </c>
-      <c r="B7" s="4" t="b">
+      <c r="B8" s="4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -932,11 +942,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="41" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -954,7 +964,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>scheduled_backups</t>
+          <t>zone_protection_enabled</t>
         </is>
       </c>
       <c r="B2" s="4" t="b">
@@ -964,39 +974,71 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>versioned_configs</t>
+          <t>dos_protection_enabled</t>
         </is>
       </c>
       <c r="B3" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>last_backup</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>restore_tested</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>job_output</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>&lt;Element 'response' at 0x7c651f7f38d0&gt;</t>
-        </is>
+          <t>packet_attack_protection</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>scheduled_backups</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>versioned_configs</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1017,7 +1059,7 @@
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="27" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
@@ -1082,7 +1124,7 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>10.2.10-h9</t>
+          <t>10.2.3</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -1102,12 +1144,12 @@
           <t>PA-02</t>
         </is>
       </c>
-      <c r="B3" s="17" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="C3" s="18" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
@@ -1119,7 +1161,7 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -1138,9 +1180,9 @@
           <t>PA-03</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>COMPLIANT</t>
         </is>
       </c>
       <c r="C4" s="16" t="inlineStr">
@@ -1155,7 +1197,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -1175,9 +1217,9 @@
           <t>PA-04</t>
         </is>
       </c>
-      <c r="B5" s="17" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>COMPLIANT</t>
         </is>
       </c>
       <c r="C5" s="16" t="inlineStr">
@@ -1192,7 +1234,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -1212,7 +1254,7 @@
           <t>PA-06</t>
         </is>
       </c>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>COMPLIANT</t>
         </is>
@@ -1229,7 +1271,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>43.8</t>
+          <t>62</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -1249,12 +1291,12 @@
           <t>PA-07</t>
         </is>
       </c>
-      <c r="B7" s="19" t="inlineStr">
-        <is>
-          <t>COMPLIANT</t>
-        </is>
-      </c>
-      <c r="C7" s="18" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
@@ -1266,7 +1308,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>0.0001</t>
+          <t>84</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -1286,7 +1328,7 @@
           <t>PA-08</t>
         </is>
       </c>
-      <c r="B8" s="19" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>COMPLIANT</t>
         </is>
@@ -1303,7 +1345,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>28.41</t>
+          <t>71</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -1323,12 +1365,12 @@
           <t>PA-10</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="C9" s="20" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>COMPLIANT</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -1340,7 +1382,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>55</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -1360,12 +1402,12 @@
           <t>PA-11</t>
         </is>
       </c>
-      <c r="B10" s="19" t="inlineStr">
-        <is>
-          <t>COMPLIANT</t>
-        </is>
-      </c>
-      <c r="C10" s="18" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
@@ -1377,7 +1419,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -1396,9 +1438,9 @@
           <t>PA-12</t>
         </is>
       </c>
-      <c r="B11" s="17" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
         </is>
       </c>
       <c r="C11" s="16" t="inlineStr">
@@ -1413,7 +1455,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>unsynchronized</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -1432,9 +1474,9 @@
           <t>PA-15</t>
         </is>
       </c>
-      <c r="B12" s="17" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>COMPLIANT</t>
         </is>
       </c>
       <c r="C12" s="16" t="inlineStr">
@@ -1449,7 +1491,7 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>True</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -1473,7 +1515,7 @@
           <t>NON_COMPLIANT</t>
         </is>
       </c>
-      <c r="C13" s="18" t="inlineStr">
+      <c r="C13" s="17" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
@@ -1485,7 +1527,7 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -1509,7 +1551,7 @@
           <t>NON_COMPLIANT</t>
         </is>
       </c>
-      <c r="C14" s="20" t="inlineStr">
+      <c r="C14" s="19" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -1521,7 +1563,7 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>18</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -1546,7 +1588,7 @@
           <t>NON_COMPLIANT</t>
         </is>
       </c>
-      <c r="C15" s="20" t="inlineStr">
+      <c r="C15" s="19" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -1558,7 +1600,7 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>25.0</t>
+          <t>40</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -1578,7 +1620,7 @@
           <t>PA-19</t>
         </is>
       </c>
-      <c r="B16" s="19" t="inlineStr">
+      <c r="B16" s="18" t="inlineStr">
         <is>
           <t>COMPLIANT</t>
         </is>
@@ -1631,7 +1673,7 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>25.0</t>
+          <t>55</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1656,7 +1698,7 @@
           <t>NON_COMPLIANT</t>
         </is>
       </c>
-      <c r="C18" s="20" t="inlineStr">
+      <c r="C18" s="19" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -1668,7 +1710,7 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1692,7 +1734,7 @@
           <t>NON_COMPLIANT</t>
         </is>
       </c>
-      <c r="C19" s="18" t="inlineStr">
+      <c r="C19" s="17" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
@@ -1728,7 +1770,7 @@
           <t>NON_COMPLIANT</t>
         </is>
       </c>
-      <c r="C20" s="18" t="inlineStr">
+      <c r="C20" s="17" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
@@ -1759,9 +1801,9 @@
           <t>PA-27</t>
         </is>
       </c>
-      <c r="B21" s="15" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>COMPLIANT</t>
         </is>
       </c>
       <c r="C21" s="16" t="inlineStr">
@@ -1776,7 +1818,7 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1795,9 +1837,9 @@
           <t>PA-28</t>
         </is>
       </c>
-      <c r="B22" s="15" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>COMPLIANT</t>
         </is>
       </c>
       <c r="C22" s="16" t="inlineStr">
@@ -1812,7 +1854,7 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1872,7 +1914,7 @@
           <t>NON_COMPLIANT</t>
         </is>
       </c>
-      <c r="C24" s="18" t="inlineStr">
+      <c r="C24" s="17" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
@@ -1903,9 +1945,9 @@
           <t>PA-34</t>
         </is>
       </c>
-      <c r="B25" s="17" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
+      <c r="B25" s="15" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
         </is>
       </c>
       <c r="C25" s="16" t="inlineStr">
@@ -1920,7 +1962,7 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -1945,7 +1987,7 @@
           <t>NON_COMPLIANT</t>
         </is>
       </c>
-      <c r="C26" s="18" t="inlineStr">
+      <c r="C26" s="17" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
@@ -1977,12 +2019,12 @@
           <t>PA-40</t>
         </is>
       </c>
-      <c r="B27" s="17" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="C27" s="20" t="inlineStr">
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>COMPLIANT</t>
+        </is>
+      </c>
+      <c r="C27" s="19" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -1994,7 +2036,7 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -2030,7 +2072,7 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -2054,7 +2096,7 @@
           <t>NON_COMPLIANT</t>
         </is>
       </c>
-      <c r="C29" s="18" t="inlineStr">
+      <c r="C29" s="17" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
@@ -2085,12 +2127,12 @@
           <t>PA-45</t>
         </is>
       </c>
-      <c r="B30" s="15" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="C30" s="20" t="inlineStr">
+      <c r="B30" s="18" t="inlineStr">
+        <is>
+          <t>COMPLIANT</t>
+        </is>
+      </c>
+      <c r="C30" s="19" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2102,7 +2144,7 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -2121,9 +2163,9 @@
           <t>PA-48</t>
         </is>
       </c>
-      <c r="B31" s="17" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
+      <c r="B31" s="15" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
         </is>
       </c>
       <c r="C31" s="16" t="inlineStr">
@@ -2138,7 +2180,7 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>False</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -2193,9 +2235,9 @@
           <t>PA-50</t>
         </is>
       </c>
-      <c r="B33" s="17" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
+      <c r="B33" s="15" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
         </is>
       </c>
       <c r="C33" s="16" t="inlineStr">
@@ -2210,7 +2252,7 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>30</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -2230,12 +2272,12 @@
           <t>PA-53</t>
         </is>
       </c>
-      <c r="B34" s="17" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="C34" s="18" t="inlineStr">
+      <c r="B34" s="15" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="C34" s="17" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
@@ -2247,7 +2289,7 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>False</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -2266,12 +2308,12 @@
           <t>PA-55</t>
         </is>
       </c>
-      <c r="B35" s="19" t="inlineStr">
+      <c r="B35" s="18" t="inlineStr">
         <is>
           <t>COMPLIANT</t>
         </is>
       </c>
-      <c r="C35" s="18" t="inlineStr">
+      <c r="C35" s="17" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
@@ -2302,12 +2344,12 @@
           <t>PA-56</t>
         </is>
       </c>
-      <c r="B36" s="17" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="C36" s="18" t="inlineStr">
+      <c r="B36" s="15" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="C36" s="17" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
@@ -2319,7 +2361,7 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>False</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -2338,12 +2380,12 @@
           <t>PA-57</t>
         </is>
       </c>
-      <c r="B37" s="17" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="C37" s="20" t="inlineStr">
+      <c r="B37" s="15" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="C37" s="19" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2355,7 +2397,7 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>45</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
@@ -2375,12 +2417,12 @@
           <t>PA-58</t>
         </is>
       </c>
-      <c r="B38" s="17" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="C38" s="20" t="inlineStr">
+      <c r="B38" s="18" t="inlineStr">
+        <is>
+          <t>COMPLIANT</t>
+        </is>
+      </c>
+      <c r="C38" s="19" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2392,7 +2434,7 @@
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
@@ -2412,9 +2454,9 @@
           <t>PA-59</t>
         </is>
       </c>
-      <c r="B39" s="17" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
+      <c r="B39" s="15" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
         </is>
       </c>
       <c r="C39" s="16" t="inlineStr">
@@ -2429,7 +2471,7 @@
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>v2c</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
@@ -2484,9 +2526,9 @@
           <t>PA-61</t>
         </is>
       </c>
-      <c r="B41" s="17" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
+      <c r="B41" s="15" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
         </is>
       </c>
       <c r="C41" s="16" t="inlineStr">
@@ -2501,7 +2543,7 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>False</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
@@ -2520,9 +2562,9 @@
           <t>PA-62</t>
         </is>
       </c>
-      <c r="B42" s="17" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
+      <c r="B42" s="18" t="inlineStr">
+        <is>
+          <t>COMPLIANT</t>
         </is>
       </c>
       <c r="C42" s="16" t="inlineStr">
@@ -2537,7 +2579,7 @@
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>True</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
@@ -2556,12 +2598,12 @@
           <t>PA-63</t>
         </is>
       </c>
-      <c r="B43" s="17" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="C43" s="20" t="inlineStr">
+      <c r="B43" s="18" t="inlineStr">
+        <is>
+          <t>COMPLIANT</t>
+        </is>
+      </c>
+      <c r="C43" s="19" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2573,7 +2615,7 @@
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>True</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
@@ -2597,7 +2639,7 @@
           <t>NON_COMPLIANT</t>
         </is>
       </c>
-      <c r="C44" s="18" t="inlineStr">
+      <c r="C44" s="17" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
@@ -2628,12 +2670,12 @@
           <t>PA-67</t>
         </is>
       </c>
-      <c r="B45" s="15" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="C45" s="20" t="inlineStr">
+      <c r="B45" s="18" t="inlineStr">
+        <is>
+          <t>COMPLIANT</t>
+        </is>
+      </c>
+      <c r="C45" s="19" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2645,7 +2687,7 @@
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
@@ -2670,14 +2712,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="27" customWidth="1" min="6" max="6"/>
     <col width="46" customWidth="1" min="7" max="7"/>
     <col width="46" customWidth="1" min="8" max="8"/>
@@ -2726,1603 +2768,1183 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="21" t="inlineStr">
+      <c r="A2" s="20" t="inlineStr">
         <is>
           <t>PA-01</t>
         </is>
       </c>
-      <c r="B2" s="22" t="inlineStr">
+      <c r="B2" s="21" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C2" s="21" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="D2" s="21" t="inlineStr">
+      <c r="C2" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D2" s="20" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
-      <c r="E2" s="21" t="inlineStr">
-        <is>
-          <t>10.2.10-h9</t>
-        </is>
-      </c>
-      <c r="F2" s="21" t="inlineStr">
+      <c r="E2" s="20" t="inlineStr">
+        <is>
+          <t>10.2.3</t>
+        </is>
+      </c>
+      <c r="F2" s="20" t="inlineStr">
         <is>
           <t>['11.1', '11.2', '12.1']</t>
         </is>
       </c>
-      <c r="G2" s="21" t="inlineStr">
-        <is>
-          <t>Observed value '10.2.10-h9' does not meet expected baseline '['11.1', '11.2', '12.1']'.</t>
-        </is>
-      </c>
-      <c r="H2" s="21" t="inlineStr">
+      <c r="G2" s="20" t="inlineStr">
+        <is>
+          <t>Observed value '10.2.3' does not meet expected baseline '['11.1', '11.2', '12.1']'.</t>
+        </is>
+      </c>
+      <c r="H2" s="20" t="inlineStr">
         <is>
           <t>Upgrade to a supported PAN-OS release.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="21" t="inlineStr">
+      <c r="A3" s="20" t="inlineStr">
         <is>
           <t>PA-02</t>
         </is>
       </c>
-      <c r="B3" s="23" t="inlineStr">
+      <c r="B3" s="22" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
       </c>
-      <c r="C3" s="21" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="D3" s="21" t="inlineStr">
+      <c r="C3" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D3" s="20" t="inlineStr">
         <is>
           <t>critical_cves</t>
         </is>
       </c>
-      <c r="E3" s="21" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F3" s="21" t="inlineStr">
+      <c r="E3" s="20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F3" s="20" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G3" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'None' does not meet expected baseline '0'.</t>
-        </is>
-      </c>
-      <c r="H3" s="21" t="inlineStr">
+      <c r="G3" s="20" t="inlineStr">
+        <is>
+          <t>Observed value '3' does not meet expected baseline '0'.</t>
+        </is>
+      </c>
+      <c r="H3" s="20" t="inlineStr">
         <is>
           <t>Apply security patches to address reported CVEs.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="21" t="inlineStr">
-        <is>
-          <t>PA-03</t>
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>PA-07</t>
         </is>
       </c>
       <c r="B4" s="22" t="inlineStr">
         <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>session_utilization</t>
+        </is>
+      </c>
+      <c r="E4" s="20" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="F4" s="20" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="G4" s="20" t="inlineStr">
+        <is>
+          <t>Observed value '84' does not meet expected baseline '80'.</t>
+        </is>
+      </c>
+      <c r="H4" s="20" t="inlineStr">
+        <is>
+          <t>Review session usage and increase capacity if needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>PA-11</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>ha_enabled</t>
+        </is>
+      </c>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F5" s="20" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G5" s="20" t="inlineStr">
+        <is>
+          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
+        </is>
+      </c>
+      <c r="H5" s="20" t="inlineStr">
+        <is>
+          <t>Enable HA and verify peer connectivity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>PA-12</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C4" s="21" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="D4" s="21" t="inlineStr">
-        <is>
-          <t>content_update_hours</t>
-        </is>
-      </c>
-      <c r="E4" s="21" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F4" s="21" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="G4" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'None' does not meet expected baseline '24'.</t>
-        </is>
-      </c>
-      <c r="H4" s="21" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="inlineStr">
+        <is>
+          <t>config_sync</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>unsynchronized</t>
+        </is>
+      </c>
+      <c r="F6" s="20" t="inlineStr">
+        <is>
+          <t>synchronized</t>
+        </is>
+      </c>
+      <c r="G6" s="20" t="inlineStr">
+        <is>
+          <t>Observed value 'unsynchronized' does not meet expected baseline 'synchronized'.</t>
+        </is>
+      </c>
+      <c r="H6" s="20" t="inlineStr">
+        <is>
+          <t>Restore HA synchronization between peers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>PA-16</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="inlineStr">
+        <is>
+          <t>any_any_rules</t>
+        </is>
+      </c>
+      <c r="E7" s="20" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F7" s="20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G7" s="20" t="inlineStr">
+        <is>
+          <t>Observed value '12' does not meet expected baseline '0'.</t>
+        </is>
+      </c>
+      <c r="H7" s="20" t="inlineStr">
+        <is>
+          <t>Remove Any-Any rules or apply strict security profiles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>PA-17</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>unused_rule_percent</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="F8" s="20" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G8" s="20" t="inlineStr">
+        <is>
+          <t>Observed value '18' does not meet expected baseline '5'.</t>
+        </is>
+      </c>
+      <c r="H8" s="20" t="inlineStr">
+        <is>
+          <t>Review and remove unused security rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>PA-18</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>documented_rule_percent</t>
+        </is>
+      </c>
+      <c r="E9" s="20" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F9" s="20" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G9" s="20" t="inlineStr">
+        <is>
+          <t>Observed value '40' does not meet expected baseline '100'.</t>
+        </is>
+      </c>
+      <c r="H9" s="20" t="inlineStr">
+        <is>
+          <t>Document all security rules with descriptions and ownership.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>PA-21</t>
+        </is>
+      </c>
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>appid_rule_percent</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="F10" s="20" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="G10" s="20" t="inlineStr">
+        <is>
+          <t>Observed value '55' does not meet expected baseline '90'.</t>
+        </is>
+      </c>
+      <c r="H10" s="20" t="inlineStr">
+        <is>
+          <t>Increase App-ID usage and reduce application=any rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>PA-23</t>
+        </is>
+      </c>
+      <c r="B11" s="23" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C11" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D11" s="20" t="inlineStr">
+        <is>
+          <t>shadowed_rules</t>
+        </is>
+      </c>
+      <c r="E11" s="20" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F11" s="20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G11" s="20" t="inlineStr">
+        <is>
+          <t>Observed value '4' does not meet expected baseline '0'.</t>
+        </is>
+      </c>
+      <c r="H11" s="20" t="inlineStr">
+        <is>
+          <t>Review shadowed rules and optimize rule order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>PA-24</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="C12" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D12" s="20" t="inlineStr">
+        <is>
+          <t>threat_prevention</t>
+        </is>
+      </c>
+      <c r="E12" s="20" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F12" s="20" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G12" s="20" t="inlineStr">
+        <is>
+          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
+        </is>
+      </c>
+      <c r="H12" s="20" t="inlineStr">
+        <is>
+          <t>Enable Threat Prevention and apply profiles to all allow rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>PA-26</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D13" s="20" t="inlineStr">
+        <is>
+          <t>dns_sinkhole_enabled</t>
+        </is>
+      </c>
+      <c r="E13" s="20" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F13" s="20" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G13" s="20" t="inlineStr">
+        <is>
+          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
+        </is>
+      </c>
+      <c r="H13" s="20" t="inlineStr">
+        <is>
+          <t>Enable DNS sinkhole for Anti-Spyware protection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>PA-29</t>
+        </is>
+      </c>
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C14" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D14" s="20" t="inlineStr">
+        <is>
+          <t>dns_security_enabled</t>
+        </is>
+      </c>
+      <c r="E14" s="20" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F14" s="20" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G14" s="20" t="inlineStr">
+        <is>
+          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
+        </is>
+      </c>
+      <c r="H14" s="20" t="inlineStr">
+        <is>
+          <t>Enable DNS Security service.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>PA-31</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="C15" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D15" s="20" t="inlineStr">
+        <is>
+          <t>ssl_decryption_enabled</t>
+        </is>
+      </c>
+      <c r="E15" s="20" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F15" s="20" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G15" s="20" t="inlineStr">
+        <is>
+          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
+        </is>
+      </c>
+      <c r="H15" s="20" t="inlineStr">
+        <is>
+          <t>Implement SSL decryption policy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>PA-34</t>
+        </is>
+      </c>
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D16" s="20" t="inlineStr">
+        <is>
+          <t>tls_minimum_version</t>
+        </is>
+      </c>
+      <c r="E16" s="20" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F16" s="20" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="G16" s="20" t="inlineStr">
+        <is>
+          <t>Observed value '1.1' does not meet expected baseline '1.2'.</t>
+        </is>
+      </c>
+      <c r="H16" s="20" t="inlineStr">
         <is>
           <t>Review configuration and align with security baseline.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="21" t="inlineStr">
-        <is>
-          <t>PA-04</t>
-        </is>
-      </c>
-      <c r="B5" s="22" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="20" t="inlineStr">
+        <is>
+          <t>PA-36</t>
+        </is>
+      </c>
+      <c r="B17" s="22" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D17" s="20" t="inlineStr">
+        <is>
+          <t>zone_count</t>
+        </is>
+      </c>
+      <c r="E17" s="20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F17" s="20" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G17" s="20" t="inlineStr">
+        <is>
+          <t>Observed value '3' does not meet expected baseline '4'.</t>
+        </is>
+      </c>
+      <c r="H17" s="20" t="inlineStr">
+        <is>
+          <t>Implement additional network segmentation zones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>PA-42</t>
+        </is>
+      </c>
+      <c r="B18" s="21" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C5" s="21" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="D5" s="21" t="inlineStr">
-        <is>
-          <t>wildfire_update_minutes</t>
-        </is>
-      </c>
-      <c r="E5" s="21" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F5" s="21" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G5" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'None' does not meet expected baseline '5'.</t>
-        </is>
-      </c>
-      <c r="H5" s="21" t="inlineStr">
-        <is>
-          <t>Review configuration and align with security baseline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="21" t="inlineStr">
-        <is>
-          <t>PA-10</t>
-        </is>
-      </c>
-      <c r="B6" s="24" t="inlineStr">
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D18" s="20" t="inlineStr">
+        <is>
+          <t>route_leaks</t>
+        </is>
+      </c>
+      <c r="E18" s="20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F18" s="20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G18" s="20" t="inlineStr">
+        <is>
+          <t>Observed value '1' does not meet expected baseline '0'.</t>
+        </is>
+      </c>
+      <c r="H18" s="20" t="inlineStr">
+        <is>
+          <t>Review routing table and remove route leakage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>PA-43</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="C19" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D19" s="20" t="inlineStr">
+        <is>
+          <t>mfa_enabled</t>
+        </is>
+      </c>
+      <c r="E19" s="20" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F19" s="20" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G19" s="20" t="inlineStr">
+        <is>
+          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
+        </is>
+      </c>
+      <c r="H19" s="20" t="inlineStr">
+        <is>
+          <t>Enable MFA for all VPN users.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>PA-48</t>
+        </is>
+      </c>
+      <c r="B20" s="21" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C20" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D20" s="20" t="inlineStr">
+        <is>
+          <t>traffic_logging_enabled</t>
+        </is>
+      </c>
+      <c r="E20" s="20" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F20" s="20" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G20" s="20" t="inlineStr">
+        <is>
+          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
+        </is>
+      </c>
+      <c r="H20" s="20" t="inlineStr">
+        <is>
+          <t>Enable traffic logging on all security policies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="20" t="inlineStr">
+        <is>
+          <t>PA-49</t>
+        </is>
+      </c>
+      <c r="B21" s="21" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C21" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D21" s="20" t="inlineStr">
+        <is>
+          <t>siem_enabled</t>
+        </is>
+      </c>
+      <c r="E21" s="20" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F21" s="20" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G21" s="20" t="inlineStr">
+        <is>
+          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
+        </is>
+      </c>
+      <c r="H21" s="20" t="inlineStr">
+        <is>
+          <t>Forward logs to SIEM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="20" t="inlineStr">
+        <is>
+          <t>PA-50</t>
+        </is>
+      </c>
+      <c r="B22" s="21" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C22" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D22" s="20" t="inlineStr">
+        <is>
+          <t>retention_days</t>
+        </is>
+      </c>
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="F22" s="20" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="G22" s="20" t="inlineStr">
+        <is>
+          <t>Observed value '30' does not meet expected baseline '90'.</t>
+        </is>
+      </c>
+      <c r="H22" s="20" t="inlineStr">
+        <is>
+          <t>Increase retention period to at least 90 days.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="20" t="inlineStr">
+        <is>
+          <t>PA-53</t>
+        </is>
+      </c>
+      <c r="B23" s="22" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="C23" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D23" s="20" t="inlineStr">
+        <is>
+          <t>default_admin_disabled</t>
+        </is>
+      </c>
+      <c r="E23" s="20" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F23" s="20" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G23" s="20" t="inlineStr">
+        <is>
+          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
+        </is>
+      </c>
+      <c r="H23" s="20" t="inlineStr">
+        <is>
+          <t>Disable or secure default administrator account.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="20" t="inlineStr">
+        <is>
+          <t>PA-56</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="C24" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D24" s="20" t="inlineStr">
+        <is>
+          <t>management_acl_enabled</t>
+        </is>
+      </c>
+      <c r="E24" s="20" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F24" s="20" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G24" s="20" t="inlineStr">
+        <is>
+          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
+        </is>
+      </c>
+      <c r="H24" s="20" t="inlineStr">
+        <is>
+          <t>Restrict management access to approved networks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
+          <t>PA-57</t>
+        </is>
+      </c>
+      <c r="B25" s="23" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C6" s="21" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="D6" s="21" t="inlineStr">
-        <is>
-          <t>disk_usage</t>
-        </is>
-      </c>
-      <c r="E6" s="21" t="inlineStr">
-        <is>
-          <t>86</t>
-        </is>
-      </c>
-      <c r="F6" s="21" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
-      </c>
-      <c r="G6" s="21" t="inlineStr">
-        <is>
-          <t>Observed value '86' does not meet expected baseline '80'.</t>
-        </is>
-      </c>
-      <c r="H6" s="21" t="inlineStr">
-        <is>
-          <t>Reduce log disk usage or increase log storage.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="21" t="inlineStr">
-        <is>
-          <t>PA-12</t>
-        </is>
-      </c>
-      <c r="B7" s="22" t="inlineStr">
+      <c r="C25" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D25" s="20" t="inlineStr">
+        <is>
+          <t>admin_timeout_minutes</t>
+        </is>
+      </c>
+      <c r="E25" s="20" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="F25" s="20" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="G25" s="20" t="inlineStr">
+        <is>
+          <t>Observed value '45' does not meet expected baseline '30'.</t>
+        </is>
+      </c>
+      <c r="H25" s="20" t="inlineStr">
+        <is>
+          <t>Reduce administrator session timeout to 30 minutes or less.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t>PA-59</t>
+        </is>
+      </c>
+      <c r="B26" s="21" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C7" s="21" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="D7" s="21" t="inlineStr">
-        <is>
-          <t>config_sync</t>
-        </is>
-      </c>
-      <c r="E7" s="21" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F7" s="21" t="inlineStr">
-        <is>
-          <t>synchronized</t>
-        </is>
-      </c>
-      <c r="G7" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'None' does not meet expected baseline 'synchronized'.</t>
-        </is>
-      </c>
-      <c r="H7" s="21" t="inlineStr">
-        <is>
-          <t>Restore HA synchronization between peers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="21" t="inlineStr">
-        <is>
-          <t>PA-15</t>
-        </is>
-      </c>
-      <c r="B8" s="22" t="inlineStr">
+      <c r="C26" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D26" s="20" t="inlineStr">
+        <is>
+          <t>snmp_version</t>
+        </is>
+      </c>
+      <c r="E26" s="20" t="inlineStr">
+        <is>
+          <t>v2c</t>
+        </is>
+      </c>
+      <c r="F26" s="20" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="G26" s="20" t="inlineStr">
+        <is>
+          <t>Observed value 'v2c' does not meet expected baseline 'v3'.</t>
+        </is>
+      </c>
+      <c r="H26" s="20" t="inlineStr">
+        <is>
+          <t>Migrate to SNMPv3 and remove weaker protocols.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="20" t="inlineStr">
+        <is>
+          <t>PA-60</t>
+        </is>
+      </c>
+      <c r="B27" s="21" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C8" s="21" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="D8" s="21" t="inlineStr">
-        <is>
-          <t>link_monitoring</t>
-        </is>
-      </c>
-      <c r="E8" s="21" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F8" s="21" t="inlineStr">
+      <c r="C27" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D27" s="20" t="inlineStr">
+        <is>
+          <t>panorama_managed</t>
+        </is>
+      </c>
+      <c r="E27" s="20" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F27" s="20" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="G8" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'None' does not meet expected baseline 'True'.</t>
-        </is>
-      </c>
-      <c r="H8" s="21" t="inlineStr">
-        <is>
-          <t>Enable path and link monitoring.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="21" t="inlineStr">
-        <is>
-          <t>PA-16</t>
-        </is>
-      </c>
-      <c r="B9" s="23" t="inlineStr">
+      <c r="G27" s="20" t="inlineStr">
+        <is>
+          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
+        </is>
+      </c>
+      <c r="H27" s="20" t="inlineStr">
+        <is>
+          <t>Integrate device with Panorama.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="20" t="inlineStr">
+        <is>
+          <t>PA-61</t>
+        </is>
+      </c>
+      <c r="B28" s="21" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C28" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D28" s="20" t="inlineStr">
+        <is>
+          <t>zone_protection_enabled</t>
+        </is>
+      </c>
+      <c r="E28" s="20" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F28" s="20" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G28" s="20" t="inlineStr">
+        <is>
+          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
+        </is>
+      </c>
+      <c r="H28" s="20" t="inlineStr">
+        <is>
+          <t>Apply Zone Protection Profiles to external zones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="20" t="inlineStr">
+        <is>
+          <t>PA-64</t>
+        </is>
+      </c>
+      <c r="B29" s="22" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
       </c>
-      <c r="C9" s="21" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="D9" s="21" t="inlineStr">
-        <is>
-          <t>any_any_rules</t>
-        </is>
-      </c>
-      <c r="E9" s="21" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F9" s="21" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G9" s="21" t="inlineStr">
-        <is>
-          <t>Observed value '4' does not meet expected baseline '0'.</t>
-        </is>
-      </c>
-      <c r="H9" s="21" t="inlineStr">
-        <is>
-          <t>Remove Any-Any rules or apply strict security profiles.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="21" t="inlineStr">
-        <is>
-          <t>PA-17</t>
-        </is>
-      </c>
-      <c r="B10" s="24" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="C10" s="21" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="D10" s="21" t="inlineStr">
-        <is>
-          <t>unused_rule_percent</t>
-        </is>
-      </c>
-      <c r="E10" s="21" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="F10" s="21" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G10" s="21" t="inlineStr">
-        <is>
-          <t>Observed value '100.0' does not meet expected baseline '5'.</t>
-        </is>
-      </c>
-      <c r="H10" s="21" t="inlineStr">
-        <is>
-          <t>Review and remove unused security rules.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="21" t="inlineStr">
-        <is>
-          <t>PA-18</t>
-        </is>
-      </c>
-      <c r="B11" s="24" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="C11" s="21" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="D11" s="21" t="inlineStr">
-        <is>
-          <t>documented_rule_percent</t>
-        </is>
-      </c>
-      <c r="E11" s="21" t="inlineStr">
-        <is>
-          <t>25.0</t>
-        </is>
-      </c>
-      <c r="F11" s="21" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="G11" s="21" t="inlineStr">
-        <is>
-          <t>Observed value '25.0' does not meet expected baseline '100'.</t>
-        </is>
-      </c>
-      <c r="H11" s="21" t="inlineStr">
-        <is>
-          <t>Document all security rules with descriptions and ownership.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="21" t="inlineStr">
-        <is>
-          <t>PA-21</t>
-        </is>
-      </c>
-      <c r="B12" s="22" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="C12" s="21" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="D12" s="21" t="inlineStr">
-        <is>
-          <t>appid_rule_percent</t>
-        </is>
-      </c>
-      <c r="E12" s="21" t="inlineStr">
-        <is>
-          <t>25.0</t>
-        </is>
-      </c>
-      <c r="F12" s="21" t="inlineStr">
-        <is>
-          <t>90</t>
-        </is>
-      </c>
-      <c r="G12" s="21" t="inlineStr">
-        <is>
-          <t>Observed value '25.0' does not meet expected baseline '90'.</t>
-        </is>
-      </c>
-      <c r="H12" s="21" t="inlineStr">
-        <is>
-          <t>Increase App-ID usage and reduce application=any rules.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="21" t="inlineStr">
-        <is>
-          <t>PA-23</t>
-        </is>
-      </c>
-      <c r="B13" s="24" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="C13" s="21" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="D13" s="21" t="inlineStr">
-        <is>
-          <t>shadowed_rules</t>
-        </is>
-      </c>
-      <c r="E13" s="21" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="F13" s="21" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G13" s="21" t="inlineStr">
-        <is>
-          <t>Observed value '6' does not meet expected baseline '0'.</t>
-        </is>
-      </c>
-      <c r="H13" s="21" t="inlineStr">
-        <is>
-          <t>Review shadowed rules and optimize rule order.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="21" t="inlineStr">
-        <is>
-          <t>PA-24</t>
-        </is>
-      </c>
-      <c r="B14" s="23" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-      <c r="C14" s="21" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="D14" s="21" t="inlineStr">
-        <is>
-          <t>threat_prevention</t>
-        </is>
-      </c>
-      <c r="E14" s="21" t="inlineStr">
+      <c r="C29" s="20" t="inlineStr">
+        <is>
+          <t>NON_COMPLIANT</t>
+        </is>
+      </c>
+      <c r="D29" s="20" t="inlineStr">
+        <is>
+          <t>scheduled_backups</t>
+        </is>
+      </c>
+      <c r="E29" s="20" t="inlineStr">
         <is>
           <t>False</t>
         </is>
       </c>
-      <c r="F14" s="21" t="inlineStr">
+      <c r="F29" s="20" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="G14" s="21" t="inlineStr">
+      <c r="G29" s="20" t="inlineStr">
         <is>
           <t>Observed value 'False' does not meet expected baseline 'True'.</t>
         </is>
       </c>
-      <c r="H14" s="21" t="inlineStr">
-        <is>
-          <t>Enable Threat Prevention and apply profiles to all allow rules.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="21" t="inlineStr">
-        <is>
-          <t>PA-26</t>
-        </is>
-      </c>
-      <c r="B15" s="23" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-      <c r="C15" s="21" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="D15" s="21" t="inlineStr">
-        <is>
-          <t>dns_sinkhole_enabled</t>
-        </is>
-      </c>
-      <c r="E15" s="21" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="F15" s="21" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="G15" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
-        </is>
-      </c>
-      <c r="H15" s="21" t="inlineStr">
-        <is>
-          <t>Enable DNS sinkhole for Anti-Spyware protection.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="21" t="inlineStr">
-        <is>
-          <t>PA-27</t>
-        </is>
-      </c>
-      <c r="B16" s="22" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="C16" s="21" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="D16" s="21" t="inlineStr">
-        <is>
-          <t>wildfire_enabled</t>
-        </is>
-      </c>
-      <c r="E16" s="21" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="F16" s="21" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="G16" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
-        </is>
-      </c>
-      <c r="H16" s="21" t="inlineStr">
-        <is>
-          <t>Enable WildFire and file forwarding.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="21" t="inlineStr">
-        <is>
-          <t>PA-28</t>
-        </is>
-      </c>
-      <c r="B17" s="22" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="C17" s="21" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="D17" s="21" t="inlineStr">
-        <is>
-          <t>url_filtering_enabled</t>
-        </is>
-      </c>
-      <c r="E17" s="21" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="F17" s="21" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="G17" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
-        </is>
-      </c>
-      <c r="H17" s="21" t="inlineStr">
-        <is>
-          <t>Enable URL Filtering and block malicious categories.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="21" t="inlineStr">
-        <is>
-          <t>PA-29</t>
-        </is>
-      </c>
-      <c r="B18" s="22" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="C18" s="21" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="D18" s="21" t="inlineStr">
-        <is>
-          <t>dns_security_enabled</t>
-        </is>
-      </c>
-      <c r="E18" s="21" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="F18" s="21" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="G18" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
-        </is>
-      </c>
-      <c r="H18" s="21" t="inlineStr">
-        <is>
-          <t>Enable DNS Security service.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="21" t="inlineStr">
-        <is>
-          <t>PA-31</t>
-        </is>
-      </c>
-      <c r="B19" s="23" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-      <c r="C19" s="21" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="D19" s="21" t="inlineStr">
-        <is>
-          <t>ssl_decryption_enabled</t>
-        </is>
-      </c>
-      <c r="E19" s="21" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="F19" s="21" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="G19" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
-        </is>
-      </c>
-      <c r="H19" s="21" t="inlineStr">
-        <is>
-          <t>Implement SSL decryption policy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="21" t="inlineStr">
-        <is>
-          <t>PA-34</t>
-        </is>
-      </c>
-      <c r="B20" s="22" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="C20" s="21" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="D20" s="21" t="inlineStr">
-        <is>
-          <t>tls_minimum_version</t>
-        </is>
-      </c>
-      <c r="E20" s="21" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F20" s="21" t="inlineStr">
-        <is>
-          <t>1.2</t>
-        </is>
-      </c>
-      <c r="G20" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'None' does not meet expected baseline '1.2'.</t>
-        </is>
-      </c>
-      <c r="H20" s="21" t="inlineStr">
-        <is>
-          <t>Review configuration and align with security baseline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="21" t="inlineStr">
-        <is>
-          <t>PA-36</t>
-        </is>
-      </c>
-      <c r="B21" s="23" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-      <c r="C21" s="21" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="D21" s="21" t="inlineStr">
-        <is>
-          <t>zone_count</t>
-        </is>
-      </c>
-      <c r="E21" s="21" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F21" s="21" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="G21" s="21" t="inlineStr">
-        <is>
-          <t>Observed value '3' does not meet expected baseline '4'.</t>
-        </is>
-      </c>
-      <c r="H21" s="21" t="inlineStr">
-        <is>
-          <t>Implement additional network segmentation zones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="21" t="inlineStr">
-        <is>
-          <t>PA-40</t>
-        </is>
-      </c>
-      <c r="B22" s="24" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="C22" s="21" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="D22" s="21" t="inlineStr">
-        <is>
-          <t>stale_nat_rules</t>
-        </is>
-      </c>
-      <c r="E22" s="21" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F22" s="21" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G22" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'None' does not meet expected baseline '0'.</t>
-        </is>
-      </c>
-      <c r="H22" s="21" t="inlineStr">
-        <is>
-          <t>Review configuration and align with security baseline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="21" t="inlineStr">
-        <is>
-          <t>PA-42</t>
-        </is>
-      </c>
-      <c r="B23" s="22" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="C23" s="21" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="D23" s="21" t="inlineStr">
-        <is>
-          <t>route_leaks</t>
-        </is>
-      </c>
-      <c r="E23" s="21" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="F23" s="21" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G23" s="21" t="inlineStr">
-        <is>
-          <t>Observed value '[]' does not meet expected baseline '0'.</t>
-        </is>
-      </c>
-      <c r="H23" s="21" t="inlineStr">
-        <is>
-          <t>Review routing table and remove route leakage.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="21" t="inlineStr">
-        <is>
-          <t>PA-43</t>
-        </is>
-      </c>
-      <c r="B24" s="23" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-      <c r="C24" s="21" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="D24" s="21" t="inlineStr">
-        <is>
-          <t>mfa_enabled</t>
-        </is>
-      </c>
-      <c r="E24" s="21" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="F24" s="21" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="G24" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
-        </is>
-      </c>
-      <c r="H24" s="21" t="inlineStr">
-        <is>
-          <t>Enable MFA for all VPN users.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="21" t="inlineStr">
-        <is>
-          <t>PA-45</t>
-        </is>
-      </c>
-      <c r="B25" s="24" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="C25" s="21" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="D25" s="21" t="inlineStr">
-        <is>
-          <t>tunnel_monitoring</t>
-        </is>
-      </c>
-      <c r="E25" s="21" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="F25" s="21" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="G25" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
-        </is>
-      </c>
-      <c r="H25" s="21" t="inlineStr">
-        <is>
-          <t>Enable VPN tunnel monitoring.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="21" t="inlineStr">
-        <is>
-          <t>PA-48</t>
-        </is>
-      </c>
-      <c r="B26" s="22" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="C26" s="21" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="D26" s="21" t="inlineStr">
-        <is>
-          <t>traffic_logging_enabled</t>
-        </is>
-      </c>
-      <c r="E26" s="21" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F26" s="21" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="G26" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'None' does not meet expected baseline 'True'.</t>
-        </is>
-      </c>
-      <c r="H26" s="21" t="inlineStr">
-        <is>
-          <t>Enable traffic logging on all security policies.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="21" t="inlineStr">
-        <is>
-          <t>PA-49</t>
-        </is>
-      </c>
-      <c r="B27" s="22" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="C27" s="21" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="D27" s="21" t="inlineStr">
-        <is>
-          <t>siem_enabled</t>
-        </is>
-      </c>
-      <c r="E27" s="21" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="F27" s="21" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="G27" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
-        </is>
-      </c>
-      <c r="H27" s="21" t="inlineStr">
-        <is>
-          <t>Forward logs to SIEM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="21" t="inlineStr">
-        <is>
-          <t>PA-50</t>
-        </is>
-      </c>
-      <c r="B28" s="22" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="C28" s="21" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="D28" s="21" t="inlineStr">
-        <is>
-          <t>retention_days</t>
-        </is>
-      </c>
-      <c r="E28" s="21" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F28" s="21" t="inlineStr">
-        <is>
-          <t>90</t>
-        </is>
-      </c>
-      <c r="G28" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'None' does not meet expected baseline '90'.</t>
-        </is>
-      </c>
-      <c r="H28" s="21" t="inlineStr">
-        <is>
-          <t>Increase retention period to at least 90 days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="21" t="inlineStr">
-        <is>
-          <t>PA-53</t>
-        </is>
-      </c>
-      <c r="B29" s="23" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-      <c r="C29" s="21" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="D29" s="21" t="inlineStr">
-        <is>
-          <t>default_admin_disabled</t>
-        </is>
-      </c>
-      <c r="E29" s="21" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F29" s="21" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="G29" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'None' does not meet expected baseline 'True'.</t>
-        </is>
-      </c>
-      <c r="H29" s="21" t="inlineStr">
-        <is>
-          <t>Disable or secure default administrator account.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="21" t="inlineStr">
-        <is>
-          <t>PA-56</t>
-        </is>
-      </c>
-      <c r="B30" s="23" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-      <c r="C30" s="21" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="D30" s="21" t="inlineStr">
-        <is>
-          <t>management_acl_enabled</t>
-        </is>
-      </c>
-      <c r="E30" s="21" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F30" s="21" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="G30" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'None' does not meet expected baseline 'True'.</t>
-        </is>
-      </c>
-      <c r="H30" s="21" t="inlineStr">
-        <is>
-          <t>Restrict management access to approved networks.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="21" t="inlineStr">
-        <is>
-          <t>PA-57</t>
-        </is>
-      </c>
-      <c r="B31" s="24" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="C31" s="21" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="D31" s="21" t="inlineStr">
-        <is>
-          <t>admin_timeout_minutes</t>
-        </is>
-      </c>
-      <c r="E31" s="21" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F31" s="21" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="G31" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'None' does not meet expected baseline '30'.</t>
-        </is>
-      </c>
-      <c r="H31" s="21" t="inlineStr">
-        <is>
-          <t>Reduce administrator session timeout to 30 minutes or less.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="21" t="inlineStr">
-        <is>
-          <t>PA-58</t>
-        </is>
-      </c>
-      <c r="B32" s="24" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="C32" s="21" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="D32" s="21" t="inlineStr">
-        <is>
-          <t>ntp_server_count</t>
-        </is>
-      </c>
-      <c r="E32" s="21" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F32" s="21" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G32" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'None' does not meet expected baseline '2'.</t>
-        </is>
-      </c>
-      <c r="H32" s="21" t="inlineStr">
-        <is>
-          <t>Configure at least two NTP servers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="21" t="inlineStr">
-        <is>
-          <t>PA-59</t>
-        </is>
-      </c>
-      <c r="B33" s="22" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="C33" s="21" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="D33" s="21" t="inlineStr">
-        <is>
-          <t>snmp_version</t>
-        </is>
-      </c>
-      <c r="E33" s="21" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F33" s="21" t="inlineStr">
-        <is>
-          <t>v3</t>
-        </is>
-      </c>
-      <c r="G33" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'None' does not meet expected baseline 'v3'.</t>
-        </is>
-      </c>
-      <c r="H33" s="21" t="inlineStr">
-        <is>
-          <t>Migrate to SNMPv3 and remove weaker protocols.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="21" t="inlineStr">
-        <is>
-          <t>PA-60</t>
-        </is>
-      </c>
-      <c r="B34" s="22" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="C34" s="21" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="D34" s="21" t="inlineStr">
-        <is>
-          <t>panorama_managed</t>
-        </is>
-      </c>
-      <c r="E34" s="21" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="F34" s="21" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="G34" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
-        </is>
-      </c>
-      <c r="H34" s="21" t="inlineStr">
-        <is>
-          <t>Integrate device with Panorama.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="21" t="inlineStr">
-        <is>
-          <t>PA-61</t>
-        </is>
-      </c>
-      <c r="B35" s="22" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="C35" s="21" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="D35" s="21" t="inlineStr">
-        <is>
-          <t>zone_protection_enabled</t>
-        </is>
-      </c>
-      <c r="E35" s="21" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F35" s="21" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="G35" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'None' does not meet expected baseline 'True'.</t>
-        </is>
-      </c>
-      <c r="H35" s="21" t="inlineStr">
-        <is>
-          <t>Apply Zone Protection Profiles to external zones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="21" t="inlineStr">
-        <is>
-          <t>PA-62</t>
-        </is>
-      </c>
-      <c r="B36" s="22" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="C36" s="21" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="D36" s="21" t="inlineStr">
-        <is>
-          <t>dos_protection_enabled</t>
-        </is>
-      </c>
-      <c r="E36" s="21" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F36" s="21" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="G36" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'None' does not meet expected baseline 'True'.</t>
-        </is>
-      </c>
-      <c r="H36" s="21" t="inlineStr">
-        <is>
-          <t>Configure DoS protection policies.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="21" t="inlineStr">
-        <is>
-          <t>PA-63</t>
-        </is>
-      </c>
-      <c r="B37" s="24" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="C37" s="21" t="inlineStr">
-        <is>
-          <t>NOT_ASSESSED</t>
-        </is>
-      </c>
-      <c r="D37" s="21" t="inlineStr">
-        <is>
-          <t>packet_attack_protection</t>
-        </is>
-      </c>
-      <c r="E37" s="21" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F37" s="21" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="G37" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'None' does not meet expected baseline 'True'.</t>
-        </is>
-      </c>
-      <c r="H37" s="21" t="inlineStr">
-        <is>
-          <t>Enable packet attack protections.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="21" t="inlineStr">
-        <is>
-          <t>PA-64</t>
-        </is>
-      </c>
-      <c r="B38" s="23" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-      <c r="C38" s="21" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="D38" s="21" t="inlineStr">
-        <is>
-          <t>scheduled_backups</t>
-        </is>
-      </c>
-      <c r="E38" s="21" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="F38" s="21" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="G38" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
-        </is>
-      </c>
-      <c r="H38" s="21" t="inlineStr">
+      <c r="H29" s="20" t="inlineStr">
         <is>
           <t>Implement daily configuration backups.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="21" t="inlineStr">
-        <is>
-          <t>PA-67</t>
-        </is>
-      </c>
-      <c r="B39" s="24" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="C39" s="21" t="inlineStr">
-        <is>
-          <t>NON_COMPLIANT</t>
-        </is>
-      </c>
-      <c r="D39" s="21" t="inlineStr">
-        <is>
-          <t>versioned_configs</t>
-        </is>
-      </c>
-      <c r="E39" s="21" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="F39" s="21" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="G39" s="21" t="inlineStr">
-        <is>
-          <t>Observed value 'False' does not meet expected baseline 'True'.</t>
-        </is>
-      </c>
-      <c r="H39" s="21" t="inlineStr">
-        <is>
-          <t>Retain at least 10 configuration snapshots.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H39"/>
+  <autoFilter ref="A1:H29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4333,10 +3955,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -4355,61 +3977,83 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>cpu_usage</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="n">
-        <v>43.8</v>
+          <t>version</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>10.2.3</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>memory_usage</t>
+          <t>critical_cves</t>
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>28.41</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>active_sessions</t>
+          <t>content_update_hours</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>max_sessions</t>
+          <t>wildfire_update_minutes</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>1100000</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>session_utilization</t>
+          <t>cpu_usage</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>0.0001</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
+          <t>session_utilization</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>memory_usage</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
           <t>disk_usage</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
-        <v>86</v>
+      <c r="B9" s="4" t="n">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -4423,11 +4067,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -4449,56 +4093,30 @@
         </is>
       </c>
       <c r="B2" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>local_state</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="n"/>
+          <t>config_sync</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>unsynchronized</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>peer_state</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>config_sync</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>runtime_sync</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
           <t>link_monitoring</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>path_monitoring</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="n"/>
+      <c r="B4" s="4" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4511,7 +4129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -4543,7 +4161,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>antivirus_profile</t>
+          <t>dns_sinkhole_enabled</t>
         </is>
       </c>
       <c r="B3" s="4" t="b">
@@ -4553,27 +4171,27 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>anti_spyware_profile</t>
+          <t>wildfire_enabled</t>
         </is>
       </c>
       <c r="B4" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>dns_sinkhole_enabled</t>
+          <t>url_filtering_enabled</t>
         </is>
       </c>
       <c r="B5" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>wildfire_enabled</t>
+          <t>dns_security_enabled</t>
         </is>
       </c>
       <c r="B6" s="4" t="b">
@@ -4583,7 +4201,7 @@
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>url_filtering_enabled</t>
+          <t>ssl_decryption_enabled</t>
         </is>
       </c>
       <c r="B7" s="4" t="b">
@@ -4593,38 +4211,14 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>dns_security_enabled</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>ssl_decryption_enabled</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
           <t>tls_minimum_version</t>
         </is>
       </c>
-      <c r="B10" s="4" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>threat_exceptions</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr"/>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4637,11 +4231,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -4659,54 +4253,64 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>virtual_routers</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>VR1</t>
-        </is>
+          <t>zone_count</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>static_routes</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>{'name': 'Default_route'}, {'name': 'Cisco_Secure_Access'}, {'name': 'Cisco_Secure_Access02'}, {'name': 'Cisco_Secure_Access_03'}, {'name': 'InternalRoute'}, {'name': 'Cisco_Secure_Access_04'}</t>
-        </is>
+          <t>stale_nat_rules</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>bgp_enabled</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="b">
+          <t>route_leaks</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>ospf_enabled</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="b">
-        <v>1</v>
+          <t>virtual_routers</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>route_leaks</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr"/>
+          <t>bgp_enabled</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>ospf_enabled</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4719,7 +4323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4745,7 +4349,7 @@
         </is>
       </c>
       <c r="B2" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -4761,31 +4365,23 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>ike_gateways</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Cisco_Secure_Access01</t>
-        </is>
+          <t>tunnel_monitoring</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>ipsec_tunnels</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>tunnel_monitoring</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="b">
-        <v>0</v>
+          <t>ike_gateways</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>GP-Gateway, SiteA-IKE</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -4799,7 +4395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4821,10 +4417,12 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>syslog_servers</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr"/>
+          <t>traffic_logging_enabled</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
@@ -4839,28 +4437,12 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>email_profiles</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>snmp_enabled</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>log_forwarding_profiles</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr"/>
+          <t>retention_days</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>30</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>